<commit_message>
I included the postgrad modudules to my data
</commit_message>
<xml_diff>
--- a/Faculties/Law/Undergrad Modules Law.xlsx
+++ b/Faculties/Law/Undergrad Modules Law.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mwamb\OneDrive\Desktop\Team_6_repo\Team19\Faculties\Law\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BD7586-DD65-4623-BCEB-04B3589DD406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA53A12A-4D1C-42A1-A583-74F28C4B0ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12084" yWindow="2064" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4907,7 +4907,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>367</v>
       </c>

</xml_diff>

<commit_message>
I have included all faculties
</commit_message>
<xml_diff>
--- a/Faculties/Law/Undergrad Modules Law.xlsx
+++ b/Faculties/Law/Undergrad Modules Law.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Law/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{EA53A12A-4D1C-42A1-A583-74F28C4B0ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71DC0CB9-CCB9-4734-8571-08AFADF79716}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{EA53A12A-4D1C-42A1-A583-74F28C4B0ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EA8C5E6-29F1-4013-B247-96C1C2558310}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1856" uniqueCount="992">
   <si>
     <t>Module Code</t>
   </si>
@@ -2047,6 +2047,960 @@
   </si>
   <si>
     <t>Compensation for occupational injuries/diseases; Unemployment Insurance; workplace health/safety; pensions; retirement funds; and social assistance</t>
+  </si>
+  <si>
+    <t>ADL711</t>
+  </si>
+  <si>
+    <t>Administrative Law 711</t>
+  </si>
+  <si>
+    <t>PGDip Public Law 7711</t>
+  </si>
+  <si>
+    <t>Discuss the main principles of administrative law; evaluate administrative powers and jurisdiction; analyze administrative action as per PAJA; and apply requirements for valid administrative actions to practical scenarios.</t>
+  </si>
+  <si>
+    <t>Foundations of administrative law; PAJA; powers and jurisdiction; action and control; valid administrative action requirements; standing and procedure; and remedies.</t>
+  </si>
+  <si>
+    <t>CLL713</t>
+  </si>
+  <si>
+    <t>Constitutional Law 713</t>
+  </si>
+  <si>
+    <t>Articulate values underlying the Constitution and evaluate its principles; interpret the Constitution in hypothetical scenarios; evaluate government structure and powers; and compare the SA constitution within international contexts.</t>
+  </si>
+  <si>
+    <t>Constitutional values and principles; constitutional history; constitutional interpretation; Bill of Rights; federalism; and the separation of powers.</t>
+  </si>
+  <si>
+    <t>CRJ711</t>
+  </si>
+  <si>
+    <t>Criminal Justice Systems and Human Rights in Africa 711</t>
+  </si>
+  <si>
+    <t>Critically evaluate the intersection between criminal justice systems and human rights in Africa, specifically focusing on vulnerable groups and unusual circumstances (e.g., states of emergency and disaster).</t>
+  </si>
+  <si>
+    <t>Criminal justice systems and human rights in Africa.</t>
+  </si>
+  <si>
+    <t>ENL711</t>
+  </si>
+  <si>
+    <t>Advanced Environmental Law 711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Environmental Law and Management 7712 </t>
+  </si>
+  <si>
+    <t>Identify and critically discuss the main rules, procedures, and principles of South African Environmental Law.</t>
+  </si>
+  <si>
+    <t>South African Environmental Law.</t>
+  </si>
+  <si>
+    <t>ENL712</t>
+  </si>
+  <si>
+    <t>Environmental Governance 712</t>
+  </si>
+  <si>
+    <t>Critically discuss the nature, scope, and function of environmental governance; analyze rules, theories, and foundations in SA; and evaluate the Constitution and enabling legal framework.</t>
+  </si>
+  <si>
+    <t>Environmental governance in South Africa.</t>
+  </si>
+  <si>
+    <t>ENL713</t>
+  </si>
+  <si>
+    <t>Environmental Administrative Law 713</t>
+  </si>
+  <si>
+    <t>Critically discuss and apply Administrative Law principles to Environmental Law; evaluate administrative powers/jurisdiction; and analyze just administrative action.</t>
+  </si>
+  <si>
+    <t>Foundations and rules of Administrative Law in environmental context; Constitution (environmental right, access to info); requirements for valid action; and remedies.</t>
+  </si>
+  <si>
+    <t>ENL714</t>
+  </si>
+  <si>
+    <t>Environmental Management 714</t>
+  </si>
+  <si>
+    <t>Critically discuss principles of environmental management and their link to governance; discuss integrated management; and evaluate the rationale behind Environmental Impact Assessments.</t>
+  </si>
+  <si>
+    <t>Environmental Impact Assessment and general environmental management.</t>
+  </si>
+  <si>
+    <t>FTL711</t>
+  </si>
+  <si>
+    <t>Concepts in Fintech Law 711</t>
+  </si>
+  <si>
+    <t>PGDip Fintech Law and Regulation 7702</t>
+  </si>
+  <si>
+    <t>Consult the Centre for African Fintech, Innovation and Law (CAFIL) for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Introduction to concepts in Fintech Law.</t>
+  </si>
+  <si>
+    <t>FTL712</t>
+  </si>
+  <si>
+    <t>Banking and Financial Regulation 712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Fintech Law and Regulation 7702 </t>
+  </si>
+  <si>
+    <t>Banking system; virtual currencies, cryptocurrencies, and central bank digital currencies; and mobile money/financial inclusion.</t>
+  </si>
+  <si>
+    <t>FTL713</t>
+  </si>
+  <si>
+    <t>Fintech Payment Regulation 713</t>
+  </si>
+  <si>
+    <t>Distinguish between payment systems regulation and oversight; and critically discuss and evaluate the meaning and legal nature of fintech payments.</t>
+  </si>
+  <si>
+    <t>Fintech payment regulation.</t>
+  </si>
+  <si>
+    <t>FTL714</t>
+  </si>
+  <si>
+    <t>Trade-offs in Fintech Regulation 714</t>
+  </si>
+  <si>
+    <t>Critically discuss the meaning and nature of financial inclusion and integrity; and analyze their relationship with Fintech.</t>
+  </si>
+  <si>
+    <t>Trade-offs in Fintech regulation.</t>
+  </si>
+  <si>
+    <t>MLG714</t>
+  </si>
+  <si>
+    <t>Multi-level Governance 714</t>
+  </si>
+  <si>
+    <t>Evaluate the constitution and enabling framework for multi-level government in SA; locate the system within international debates; and compare provincial government finance sources.</t>
+  </si>
+  <si>
+    <t>Power distribution between national, provincial, and local government; constitutional framework; multi-level finance; and intergovernmental relations.</t>
+  </si>
+  <si>
+    <t>LGL712</t>
+  </si>
+  <si>
+    <t>Local Government 712</t>
+  </si>
+  <si>
+    <t>Articulate the constitution and enabling framework for local government in SA; identify strategies to integrate ethics and good governance; and locate the system within international debates.</t>
+  </si>
+  <si>
+    <t>Local government.</t>
+  </si>
+  <si>
+    <t>PGL711</t>
+  </si>
+  <si>
+    <t>Labour Law in Context 711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Labour Law 7701 </t>
+  </si>
+  <si>
+    <t>Critically analyze the elements of collective bargaining (including industrial action); demonstrate ability to engage with practical requirements; and apply statutory provisions for business transfers.</t>
+  </si>
+  <si>
+    <t>Historical development of SA labour law; contract principles; the constitutional framework (LRA, BCEA, EEA); legal interpretation; and collective bargaining.</t>
+  </si>
+  <si>
+    <t>PGL712</t>
+  </si>
+  <si>
+    <t>The Right to Fair Labour Practices 712</t>
+  </si>
+  <si>
+    <t>Analyze concepts relevant to dismissal and unfair labour practices; demonstrate knowledge of constitutional/international rights; explain the role of common law; and apply SA labour legislation.</t>
+  </si>
+  <si>
+    <t>The right to fair labour practices.</t>
+  </si>
+  <si>
+    <t>PGL721</t>
+  </si>
+  <si>
+    <t>Labour Dispute Resolution 721</t>
+  </si>
+  <si>
+    <t>Consult the Mercantile and Labour Law Department for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Labour dispute resolution.</t>
+  </si>
+  <si>
+    <t>PGL722</t>
+  </si>
+  <si>
+    <t>Advanced Dispute Resolution Procedure 722</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of ethical issues in conciliation and arbitration; explain and apply conciliation process elements; and demonstrate ability to conduct conciliation.</t>
+  </si>
+  <si>
+    <t>Conciliation; con-arb; conducting arbitration; representation; duties and powers; evidence admissibility; and arbitration awards (variation, rescission, and review).</t>
+  </si>
+  <si>
+    <t>PUB711</t>
+  </si>
+  <si>
+    <t>Detention and Oversight 711</t>
+  </si>
+  <si>
+    <t>Consult the Dullah Omar Institute for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Detention and oversight, with specific reference to vulnerable groups and emergency/disaster situations.</t>
+  </si>
+  <si>
+    <t>TXL711</t>
+  </si>
+  <si>
+    <t>Advanced Income Tax Law 711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Tax Law 7721 </t>
+  </si>
+  <si>
+    <t>Critically analyze "gross income" and constituent elements; understand residence and "place of effective management"; interpret source rules; and solve problems in factual scenarios.</t>
+  </si>
+  <si>
+    <t>Interpretation of fiscal statutes; Constitution impact; gross income (resident/non-resident); partnerships; revenue vs capital; and taxation of cryptocurrency.</t>
+  </si>
+  <si>
+    <t>TXL712</t>
+  </si>
+  <si>
+    <t>International Tax Law 712</t>
+  </si>
+  <si>
+    <t>Critically analyze fundamental concepts in international taxation; understand OECD model conventions; interpret double tax agreements; and evaluate international transactions.</t>
+  </si>
+  <si>
+    <t>International tax law.</t>
+  </si>
+  <si>
+    <t>TXL713</t>
+  </si>
+  <si>
+    <t>Tax Administration 713</t>
+  </si>
+  <si>
+    <t>Analyze legal concepts under the TAA, PAJA, and the Constitution; explain taxpayer rights (privacy, property, access); and interpret rules governing appeals and objections.</t>
+  </si>
+  <si>
+    <t>Inter-relationship between TAA, PAJA, and the Constitution; taxpayer rights to just administrative action and court access; and appeal/objection rules.</t>
+  </si>
+  <si>
+    <t>TXL714</t>
+  </si>
+  <si>
+    <t>Estate Planning Law 714</t>
+  </si>
+  <si>
+    <t>Critically understand the concept of estate duty and its SA operation; understand the meaning of an "estate"; and explain components relevant to determining dutiable amounts.</t>
+  </si>
+  <si>
+    <t>Estate planning law.</t>
+  </si>
+  <si>
+    <t>ACL811</t>
+  </si>
+  <si>
+    <t>Anti-Corruption Law 811</t>
+  </si>
+  <si>
+    <t>LLM 7801, LLM 7821, LLM 7822</t>
+  </si>
+  <si>
+    <t>Comprehend national/international dimensions of corruption; understand corruption as a barrier to development and human rights; and recognize/assess obstacles to anti-corruption practices.</t>
+  </si>
+  <si>
+    <t>Corruption meaning and extent; forms; evolution of law; SA anti-corruption statutes/cases; prevention and prosecution; collaboration; and asset recovery.</t>
+  </si>
+  <si>
+    <t>AML811</t>
+  </si>
+  <si>
+    <t>Anti-Money Laundering Law 811</t>
+  </si>
+  <si>
+    <t>Consult the Criminal Justice and Procedure Department for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Anti-money laundering law transnationally.</t>
+  </si>
+  <si>
+    <t>CCL811</t>
+  </si>
+  <si>
+    <t>Comparative Constitutional Law 811</t>
+  </si>
+  <si>
+    <t>LLM 7801, LLM 7821, LLM 7822, MPhil 7871, MPhil 7860, MPhil 7861</t>
+  </si>
+  <si>
+    <t>Apply comparative constitutional law methodology; and critically analyze constitutions regarding organizing government, rights models, constitutional review, and reform mechanisms.</t>
+  </si>
+  <si>
+    <t>Comparative law methodologies; principles; constitution making; systems/forms of government; judicial appointment; emergency powers; and review models.</t>
+  </si>
+  <si>
+    <t>CDS811</t>
+  </si>
+  <si>
+    <t>Constitutional Design in Divided Societies 811</t>
+  </si>
+  <si>
+    <t>Evaluate how a divided society's constitution can design state institutions to manage communities; demonstrate knowledge of constitutional choices for multi-ethnic states; and analyze options for polarized societies.</t>
+  </si>
+  <si>
+    <t>Challenges of divided societies; Bill of Rights response; constitutionalism; federalism; territorial pluralism; electoral systems; and language policy.</t>
+  </si>
+  <si>
+    <t>CIN800</t>
+  </si>
+  <si>
+    <t>Constitutional Rights Interpretation 800</t>
+  </si>
+  <si>
+    <t>Analyze challenges facing rights interpretation in young democracies; understand hermeneutic/political factors; and identify and solve problems relating to specific constitutional rights.</t>
+  </si>
+  <si>
+    <t>Theories of interpretation; doctrines (separation of powers, popular constitutionalism); hermeneutic factors (text, values); and alternative theories (textualism, deconstruction).</t>
+  </si>
+  <si>
+    <t>CIN811</t>
+  </si>
+  <si>
+    <t>Constitutional Law, Politics and Theory 811</t>
+  </si>
+  <si>
+    <t>Critically evaluate the concepts and ideas central to modern constitutions; and provide in-depth research analysis of covered topics.</t>
+  </si>
+  <si>
+    <t>The concept of the ‘political’ and the ‘constitution’; sovereignty; constituent power; democracy; and contemporary problems (e.g., right to the city, decolonial perspectives).</t>
+  </si>
+  <si>
+    <t>CLL811</t>
+  </si>
+  <si>
+    <t>Constitutional Law Practice 811</t>
+  </si>
+  <si>
+    <t>Acquire an understanding of how constitutional law is applied in practice; provide legal advice/opinions on interpretation in practical situations; and solve problems using creative thinking.</t>
+  </si>
+  <si>
+    <t>Practical research in constitutional law; internship experience at an institution of democracy; and praxis of application.</t>
+  </si>
+  <si>
+    <t>CLL812</t>
+  </si>
+  <si>
+    <t>Constitutional Rights and Criminal Justice 812</t>
+  </si>
+  <si>
+    <t>Analyze fundamental concepts and principles of constitutional interpretation in criminal justice; demonstrate knowledge of the Bill of Rights; and evaluate case law.</t>
+  </si>
+  <si>
+    <t>Bill of Rights examining: privacy and police powers (search/seizure); arrest and force; detainee rights (legal services); bail; and fair trial.</t>
+  </si>
+  <si>
+    <t>CLL814</t>
+  </si>
+  <si>
+    <t>Multi-level Governance 814</t>
+  </si>
+  <si>
+    <t>Analyze fundamental legal concepts, theories, and practices of intergovernmental relations in SA; and identify and solve problems regarding dispersal of powers and supervisory reach.</t>
+  </si>
+  <si>
+    <t>Multi-level governance.</t>
+  </si>
+  <si>
+    <t>CLL815</t>
+  </si>
+  <si>
+    <t>Gender Equality and Women’s Rights 815</t>
+  </si>
+  <si>
+    <t>Critically evaluate, apply, and reflect on concepts and theories relating to substantive gender equality and women’s rights; and conduct analysis from a gender perspective.</t>
+  </si>
+  <si>
+    <t>Gender equality and women’s rights.</t>
+  </si>
+  <si>
+    <t>CLL816</t>
+  </si>
+  <si>
+    <t>Legal Pluralism 816</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822, MPhil 7871, MPhil 7860, MPhil 7861, LLM 7801, LLM 7821, LLM 7822 LPFL </t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of pluralism theories; challenge mainstream conceptualizations of customary law; explain pluralism as a product of legal history; and critique the indigenous-state law relationship.</t>
+  </si>
+  <si>
+    <t>Historical context; impact of colonial rule; major theories vs cultural relativism; customary law critique; dialogue areas between state and indigenous laws; and decolonization.</t>
+  </si>
+  <si>
+    <t>CLL817</t>
+  </si>
+  <si>
+    <t>Children’s Rights 817</t>
+  </si>
+  <si>
+    <t>Children’s rights.</t>
+  </si>
+  <si>
+    <t>CLL818</t>
+  </si>
+  <si>
+    <t>Climate Law and Governance 818</t>
+  </si>
+  <si>
+    <t>IEL812</t>
+  </si>
+  <si>
+    <t>Consult the Global Environmental Law Centre for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Climate change law and relevant governance; sectoral legislation; principles; international/SA actors; climate justice; and damages/liability.</t>
+  </si>
+  <si>
+    <t>CLL819</t>
+  </si>
+  <si>
+    <t>Constitutional Law and Nature 819</t>
+  </si>
+  <si>
+    <t>Evaluate law for protecting nature and non-human animals; analyze taxonomy of environmental constitutionalism; and understand Earth Jurisprudence/non-anthropocentric approaches.</t>
+  </si>
+  <si>
+    <t>Governance scope for environment/nature; right holders; substantive/procedural rights; and concepts (Anthropocentrism, Rule of Law, Public Trust, Rights of Nature).</t>
+  </si>
+  <si>
+    <t>CLL821</t>
+  </si>
+  <si>
+    <t>Animal Law and Rights 821</t>
+  </si>
+  <si>
+    <t>Critically evaluate the philosophical, ethical, scientific, and legal foundations of the protection of animals in South Africa and globally.</t>
+  </si>
+  <si>
+    <t>Current legal system deficiencies; core concepts (welfare, legal personhood, sentience, speciesism); and animal rights in the courts.</t>
+  </si>
+  <si>
+    <t>COR811</t>
+  </si>
+  <si>
+    <t>Corporate Governance and Remedies 811</t>
+  </si>
+  <si>
+    <t>Analyze fundamental concepts and principles of corporate governance; examine main role players; evaluate SA regulation vs international practice; and identify shortcomings/solutions.</t>
+  </si>
+  <si>
+    <t>Theories of governance; King Reports (I-IV); role players; comparative studies (CSR, Ethical Leadership, Criminal Liability); and corporate law remedies.</t>
+  </si>
+  <si>
+    <t>COR812</t>
+  </si>
+  <si>
+    <t>Corporate Financial Regulation 812</t>
+  </si>
+  <si>
+    <t>Conceptualize Approach to financial regulation (Companies Act 2008); interpret decision-making principles for corporate finance; and explain rules for market abuse prevention.</t>
+  </si>
+  <si>
+    <t>SA/international principles; funding sources (equity); capital regulation (solvency/liquidity); distributions; and policy objectives of securities/financial markets.</t>
+  </si>
+  <si>
+    <t>COR813</t>
+  </si>
+  <si>
+    <t>Corporate Insolvency Law 813</t>
+  </si>
+  <si>
+    <t>Analyze options when a company enters the zone of insolvency; explain business rescue regulation and practice; and interpret relevant case law and statutes.</t>
+  </si>
+  <si>
+    <t>Corporate solvency principles; restructuring; business rescue framework (Practitioner powers, plan, termination); liquidations; and cross-border issues.</t>
+  </si>
+  <si>
+    <t>CPL811</t>
+  </si>
+  <si>
+    <t>Constitutional Property Law 811</t>
+  </si>
+  <si>
+    <t>Demonstrate specialist knowledge of "property" (section 25); interpret regulatory control (planning, mining, neighbor law); and design alternative land reform strategies.</t>
+  </si>
+  <si>
+    <t>SA Bill of Rights (property); legal framework for regulatory control; methodological approaches; and the property relationship with other constitutional rights.</t>
+  </si>
+  <si>
+    <t>CPL812</t>
+  </si>
+  <si>
+    <t>Land Reform and Housing Law 812</t>
+  </si>
+  <si>
+    <t>Consult the Private Law Department for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>Land reform and housing law.</t>
+  </si>
+  <si>
+    <t>CPT811</t>
+  </si>
+  <si>
+    <t>Competition Law and Regulation 811</t>
+  </si>
+  <si>
+    <t>Demonstrate specialist knowledge of competition theoretical underpinnings; explain competition economics; apply rules to practical scenarios; and analyze social justice relations.</t>
+  </si>
+  <si>
+    <t>Harvard/Chicago schools; economics/structures; horizontal/vertical practices; mergers; abuse of dominance; jurisdictions; and relations with IP, information, and labour law.</t>
+  </si>
+  <si>
+    <t>CPT812</t>
+  </si>
+  <si>
+    <t>Competition Law and Work 812</t>
+  </si>
+  <si>
+    <t>Identify and critically analyze the link between competition and labour law; analyze effects of employer monopsony power; and conceptualize "platform work" impact.</t>
+  </si>
+  <si>
+    <t>General principles/economics; market structures (monopsonies); defining workers; labour rights; Competition Act scope; and transformation/digitisation.</t>
+  </si>
+  <si>
+    <t>CPT813</t>
+  </si>
+  <si>
+    <t>Mergers and Acquisitions 813</t>
+  </si>
+  <si>
+    <t>Conceptualize amalgamations/mergers and underpinning policies; interpret the legal framework (Companies Act 2008, Competition Act 1998); and explain takeover regulation.</t>
+  </si>
+  <si>
+    <t>Fundamental transactions; merger structures and effect; statutory merger procedures (Companies/Competition Acts); stakeholder protection; and the Takeover Regulation Panel.</t>
+  </si>
+  <si>
+    <t>CPT814</t>
+  </si>
+  <si>
+    <t>Competition and Information Law 814</t>
+  </si>
+  <si>
+    <t>Understand dynamic functions of a modern economy; conceptualize key areas of information law in the digital age; and critically evaluate competition in the digital economy.</t>
+  </si>
+  <si>
+    <t>Online consumer protection; privacy; computer crime; trade in digital services; AI; digital taxation; and technological approaches to enforcement in digital markets.</t>
+  </si>
+  <si>
+    <t>DLP812</t>
+  </si>
+  <si>
+    <t>Disability Law and the Workplace 812</t>
+  </si>
+  <si>
+    <t>Demonstrate a specialist knowledge of the international legal framework relating to disability and the workplace.</t>
+  </si>
+  <si>
+    <t>Disability law and the workplace.</t>
+  </si>
+  <si>
+    <t>DPR811</t>
+  </si>
+  <si>
+    <t>Dispute Resolution 811</t>
+  </si>
+  <si>
+    <t>Negotiation, mediation, and arbitration processes; SA Truth and Reconciliation Commission; and restorative justice.</t>
+  </si>
+  <si>
+    <t>ESP811</t>
+  </si>
+  <si>
+    <t>The Extension of Social Protection 811</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts of social protection.</t>
+  </si>
+  <si>
+    <t>The extension of social protection.</t>
+  </si>
+  <si>
+    <t>FAM811</t>
+  </si>
+  <si>
+    <t>International Family Law 811</t>
+  </si>
+  <si>
+    <t>Consult the Centre for Legal Integration in Africa (CLIA) for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>International family law.</t>
+  </si>
+  <si>
+    <t>IAL812</t>
+  </si>
+  <si>
+    <t>International Anti-Corruption Law 812</t>
+  </si>
+  <si>
+    <t>Appreciate the significance of corruption as an international crisis; understand it as a barrier to socio-economic development; and recognize obstacles to anti-corruption practices.</t>
+  </si>
+  <si>
+    <t>International anti-corruption law.</t>
+  </si>
+  <si>
+    <t>IEL811</t>
+  </si>
+  <si>
+    <t>International Environmental Law 811</t>
+  </si>
+  <si>
+    <t>ENV431/equiv</t>
+  </si>
+  <si>
+    <t>Evaluate what constitutes the "environment" internationally; and understand the application of international/regional policies and legal norms in SA domestic law.</t>
+  </si>
+  <si>
+    <t>IEL and SADC law pertaining to environment (SA perspective); Biodiversity; Sea/Wildlife law; Climate Change; and trade/development.</t>
+  </si>
+  <si>
+    <t>Advanced Environmental Law 812</t>
+  </si>
+  <si>
+    <t>IEL811 (pref)</t>
+  </si>
+  <si>
+    <t>Critically evaluate the "environment"; identify ethical duties; identify complex environmentally related matters; and apply specialist knowledge to address/solve them.</t>
+  </si>
+  <si>
+    <t>Environment law scope; international/human rights dimensions; administration; implementation/enforcement; and natural/cultural resource utilization.</t>
+  </si>
+  <si>
+    <t>IHR811</t>
+  </si>
+  <si>
+    <t>International Criminal Law 811</t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of international crimes; identify principles from sources to solve cases; evaluate ICC enforcement; and assess African reform/decolonisation proposals.</t>
+  </si>
+  <si>
+    <t>International criminal law.</t>
+  </si>
+  <si>
+    <t>IHR812</t>
+  </si>
+  <si>
+    <t>Transitional Justice 812</t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of meaning/origin/debates; critically analyze AU approach within decolonized context; and conduct research for transitional justice scenarios.</t>
+  </si>
+  <si>
+    <t>Research/writing; theories (amnesty, truth, commissions); international law (Human rights/humanitarian); context studies (SA, Rwanda, DRC, etc.).</t>
+  </si>
+  <si>
+    <t>IHR813</t>
+  </si>
+  <si>
+    <t>Comparative Regional Integration &amp; Dev. 813</t>
+  </si>
+  <si>
+    <t>Comparative regional integration; trade; and human rights protection.</t>
+  </si>
+  <si>
+    <t>IHR814</t>
+  </si>
+  <si>
+    <t>Int. Protection of Human Rights Law 814</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of fundamental concepts/principles/theories; and apply research methods and strategies to theoretical and applied situations.</t>
+  </si>
+  <si>
+    <t>Introduction to African, European, Inter-American, Asian, and Arab systems for human rights protection.</t>
+  </si>
+  <si>
+    <t>IHR815</t>
+  </si>
+  <si>
+    <t>International Humanitarian Law 815</t>
+  </si>
+  <si>
+    <t>Consult the African Centre for Transnational Criminal Justice for detailed outcomes.</t>
+  </si>
+  <si>
+    <t>International humanitarian law.</t>
+  </si>
+  <si>
+    <t>IHR816</t>
+  </si>
+  <si>
+    <t>Global Human Rights Issues 816</t>
+  </si>
+  <si>
+    <t>Critically analyze contemporary human rights issues; evaluate monitoring limits and politicization; and analyze links between rights, development, and poverty.</t>
+  </si>
+  <si>
+    <t>Global human rights issues.</t>
+  </si>
+  <si>
+    <t>IPL831</t>
+  </si>
+  <si>
+    <t>Intellectual Property Law 831</t>
+  </si>
+  <si>
+    <t>Critically discuss fundamental legal theories, concepts, and principles of intellectual property.</t>
+  </si>
+  <si>
+    <t>Intellectual property law.</t>
+  </si>
+  <si>
+    <t>ITB811</t>
+  </si>
+  <si>
+    <t>International Trade 811</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of concepts and principles; and apply methods and strategies involved in legal research and problem solving.</t>
+  </si>
+  <si>
+    <t>International trade law practices; international economic/trade dispute settlement (arbitration).</t>
+  </si>
+  <si>
+    <t>ITB812</t>
+  </si>
+  <si>
+    <t>International Business &amp; Regional Trade Law 812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822 7811 </t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of concepts, principles, theories, and their relationship to international business practices.</t>
+  </si>
+  <si>
+    <t>Sales, finance, and competition forms; arbitration; environmental/social considerations; EU Law; AGOA, SADC, AU roles; and African trade negotiation roles.</t>
+  </si>
+  <si>
+    <t>ITB813</t>
+  </si>
+  <si>
+    <t>International Economic &amp; Investment Law 813</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts and principles of investment law.</t>
+  </si>
+  <si>
+    <t>Public/private international law; state responsibility; treaties; global institutes (UNCTAD, AfDB, IMF); WTO regulation; IP (TRIPS); and investment regulation in Africa.</t>
+  </si>
+  <si>
+    <t>ITT811</t>
+  </si>
+  <si>
+    <t>International Taxation Law 811</t>
+  </si>
+  <si>
+    <t>Critically analyze concepts/theories of international taxation; evaluate OECD models vs SA; interpret rules for double tax agreements; and argue for decolonized principles.</t>
+  </si>
+  <si>
+    <t>Jurisdiction (source/residence); treatment of income for different taxpayers; international headquarter companies; double tax agreements; and Constitution impact.</t>
+  </si>
+  <si>
+    <t>LAB811</t>
+  </si>
+  <si>
+    <t>Labour Law in the New Global Market 811</t>
+  </si>
+  <si>
+    <t>Collective bargaining and minimum standards in non-standard employment markets; workplace equality/affirmative action; and 4IR context.</t>
+  </si>
+  <si>
+    <t>LAB812</t>
+  </si>
+  <si>
+    <t>Law of Unfair Dismissal 812</t>
+  </si>
+  <si>
+    <t>Analyze concepts, principles, and theories relevant to dismissal development; and apply research methods and strategies.</t>
+  </si>
+  <si>
+    <t>Law of unfair dismissal.</t>
+  </si>
+  <si>
+    <t>LGG811</t>
+  </si>
+  <si>
+    <t>Constitutional Governance 811</t>
+  </si>
+  <si>
+    <t>Demonstrate understanding of rule of law principles; critically discuss SA constitutionalism; evaluate SA system in international debates; and critically analyze/solve problems.</t>
+  </si>
+  <si>
+    <t>Constitutional governance; rule of law; internal/external accountability; Chapter 9 institutions; PAIA; procurement; PAJA; review; Ubuntu; and digital impact.</t>
+  </si>
+  <si>
+    <t>LGL812</t>
+  </si>
+  <si>
+    <t>Local Government 812</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts, principles, theories, and practices of local government in SA.</t>
+  </si>
+  <si>
+    <t>LPS812</t>
+  </si>
+  <si>
+    <t>Punishment and Sentencing 812</t>
+  </si>
+  <si>
+    <t>Penalty clauses in international treaties; minimum/mandatory sentences; judicial discretion; mitigation/aggravation; and Bill of Rights relationship.</t>
+  </si>
+  <si>
+    <t>OML811</t>
+  </si>
+  <si>
+    <t>Int. Anti-Money Laundering Law 811</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of how the crime of money laundering developed transnationally.</t>
+  </si>
+  <si>
+    <t>International anti-money laundering law.</t>
+  </si>
+  <si>
+    <t>PRL811</t>
+  </si>
+  <si>
+    <t>Islamic Law and Jurisprudence 811</t>
+  </si>
+  <si>
+    <t>Critically analyze schools of religious thought in Islam; assess conflict between rights approaches and scriptural interpretation; and evaluate state/non-state roles.</t>
+  </si>
+  <si>
+    <t>Muslim Personal Law.</t>
+  </si>
+  <si>
+    <t>SER811</t>
+  </si>
+  <si>
+    <t>Economic, Social and Cultural Rights 811</t>
+  </si>
+  <si>
+    <t>Understand theories relating to enforcement; apply research methods; identify international instruments/oversight bodies; and engage with separation of powers issues.</t>
+  </si>
+  <si>
+    <t>Economic, social, and cultural rights.</t>
+  </si>
+  <si>
+    <t>SIT811</t>
+  </si>
+  <si>
+    <t>Dispute Settlement in Int. Transactions 811</t>
+  </si>
+  <si>
+    <t>Demonstrate understanding of trade/investment/business transactions; evaluate conflicts; analyze settlement legitimacy based on jurisprudence; and formulate views on shortcomings.</t>
+  </si>
+  <si>
+    <t>Dispute settlement in international transactions.</t>
+  </si>
+  <si>
+    <t>TLA812</t>
+  </si>
+  <si>
+    <t>Tax Administration 812</t>
+  </si>
+  <si>
+    <t>Analyze rules under the TAA, PAJA, and the Constitution; explain taxpayer rights (privacy, property, access); and interpret rules for appeals and objections.</t>
+  </si>
+  <si>
+    <t>Provisions of TAA, PAJA, and the Constitution; inter-relationships; taxpayer rights; and court/tribunal access.</t>
+  </si>
+  <si>
+    <t>Full Thesis</t>
+  </si>
+  <si>
+    <t>Full Thesis 801 / 802</t>
+  </si>
+  <si>
+    <t>Made a satisfactory contribution to knowledge in Law or its interaction with another discipline by either proposing a significant research question or through substantial studies.</t>
+  </si>
+  <si>
+    <t>Research project in any area of Law or interaction with another field.</t>
+  </si>
+  <si>
+    <t>Mini Thesis</t>
+  </si>
+  <si>
+    <t>Mini Thesis 803 / 804</t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law or interaction with another discipline following a research question with potential.</t>
+  </si>
+  <si>
+    <t>Research proposals from any area of Law; interaction with another field; and substantial historical or comparative studies.</t>
+  </si>
+  <si>
+    <t>LPF803/4</t>
+  </si>
+  <si>
+    <t>Legal Pluralism and Family Mini Thesis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822 LPFL </t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law following a research question with satisfactory potential; carry out and report on research.</t>
+  </si>
+  <si>
+    <t>Mini-thesis in Legal Pluralism and Family Law.</t>
+  </si>
+  <si>
+    <t>Res. Paper</t>
+  </si>
+  <si>
+    <t>Research Paper 805 / 806</t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law; carry out and report on research in an approximately 18,000-word paper suitable for publication.</t>
+  </si>
+  <si>
+    <t>Research Paper.</t>
   </si>
 </sst>
 </file>
@@ -2105,7 +3059,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2113,6 +3067,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2128,6 +3083,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2393,10 +3352,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I253"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
     <col min="6" max="6" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7446,7 +8406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" ht="349.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>383</v>
       </c>
@@ -7473,6 +8433,2268 @@
       </c>
       <c r="I175" s="1">
         <v>15</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>674</v>
+      </c>
+      <c r="B176" t="s">
+        <v>675</v>
+      </c>
+      <c r="C176">
+        <v>1</v>
+      </c>
+      <c r="D176" t="s">
+        <v>676</v>
+      </c>
+      <c r="E176" t="s">
+        <v>17</v>
+      </c>
+      <c r="F176" t="s">
+        <v>17</v>
+      </c>
+      <c r="G176" t="s">
+        <v>677</v>
+      </c>
+      <c r="H176" t="s">
+        <v>678</v>
+      </c>
+      <c r="I176">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>679</v>
+      </c>
+      <c r="B177" t="s">
+        <v>680</v>
+      </c>
+      <c r="C177">
+        <v>1</v>
+      </c>
+      <c r="D177" t="s">
+        <v>676</v>
+      </c>
+      <c r="E177" t="s">
+        <v>17</v>
+      </c>
+      <c r="F177" t="s">
+        <v>17</v>
+      </c>
+      <c r="G177" t="s">
+        <v>681</v>
+      </c>
+      <c r="H177" t="s">
+        <v>682</v>
+      </c>
+      <c r="I177">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>683</v>
+      </c>
+      <c r="B178" t="s">
+        <v>684</v>
+      </c>
+      <c r="C178">
+        <v>1</v>
+      </c>
+      <c r="D178" t="s">
+        <v>676</v>
+      </c>
+      <c r="E178" t="s">
+        <v>17</v>
+      </c>
+      <c r="F178" t="s">
+        <v>17</v>
+      </c>
+      <c r="G178" t="s">
+        <v>685</v>
+      </c>
+      <c r="H178" t="s">
+        <v>686</v>
+      </c>
+      <c r="I178">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>687</v>
+      </c>
+      <c r="B179" t="s">
+        <v>688</v>
+      </c>
+      <c r="C179">
+        <v>1</v>
+      </c>
+      <c r="D179" t="s">
+        <v>689</v>
+      </c>
+      <c r="E179" t="s">
+        <v>17</v>
+      </c>
+      <c r="F179" t="s">
+        <v>17</v>
+      </c>
+      <c r="G179" t="s">
+        <v>690</v>
+      </c>
+      <c r="H179" t="s">
+        <v>691</v>
+      </c>
+      <c r="I179">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>692</v>
+      </c>
+      <c r="B180" t="s">
+        <v>693</v>
+      </c>
+      <c r="C180">
+        <v>1</v>
+      </c>
+      <c r="D180" t="s">
+        <v>689</v>
+      </c>
+      <c r="E180" t="s">
+        <v>17</v>
+      </c>
+      <c r="F180" t="s">
+        <v>17</v>
+      </c>
+      <c r="G180" t="s">
+        <v>694</v>
+      </c>
+      <c r="H180" t="s">
+        <v>695</v>
+      </c>
+      <c r="I180">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>696</v>
+      </c>
+      <c r="B181" t="s">
+        <v>697</v>
+      </c>
+      <c r="C181">
+        <v>1</v>
+      </c>
+      <c r="D181" t="s">
+        <v>689</v>
+      </c>
+      <c r="E181" t="s">
+        <v>17</v>
+      </c>
+      <c r="F181" t="s">
+        <v>17</v>
+      </c>
+      <c r="G181" t="s">
+        <v>698</v>
+      </c>
+      <c r="H181" t="s">
+        <v>699</v>
+      </c>
+      <c r="I181">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>700</v>
+      </c>
+      <c r="B182" t="s">
+        <v>701</v>
+      </c>
+      <c r="C182">
+        <v>1</v>
+      </c>
+      <c r="D182" t="s">
+        <v>689</v>
+      </c>
+      <c r="E182" t="s">
+        <v>17</v>
+      </c>
+      <c r="F182" t="s">
+        <v>17</v>
+      </c>
+      <c r="G182" t="s">
+        <v>702</v>
+      </c>
+      <c r="H182" t="s">
+        <v>703</v>
+      </c>
+      <c r="I182">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>704</v>
+      </c>
+      <c r="B183" t="s">
+        <v>705</v>
+      </c>
+      <c r="C183">
+        <v>1</v>
+      </c>
+      <c r="D183" t="s">
+        <v>706</v>
+      </c>
+      <c r="E183" t="s">
+        <v>17</v>
+      </c>
+      <c r="F183" t="s">
+        <v>17</v>
+      </c>
+      <c r="G183" t="s">
+        <v>707</v>
+      </c>
+      <c r="H183" t="s">
+        <v>708</v>
+      </c>
+      <c r="I183">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>709</v>
+      </c>
+      <c r="B184" t="s">
+        <v>710</v>
+      </c>
+      <c r="C184">
+        <v>1</v>
+      </c>
+      <c r="D184" t="s">
+        <v>711</v>
+      </c>
+      <c r="E184" t="s">
+        <v>17</v>
+      </c>
+      <c r="F184" t="s">
+        <v>17</v>
+      </c>
+      <c r="G184" t="s">
+        <v>707</v>
+      </c>
+      <c r="H184" t="s">
+        <v>712</v>
+      </c>
+      <c r="I184">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>713</v>
+      </c>
+      <c r="B185" t="s">
+        <v>714</v>
+      </c>
+      <c r="C185">
+        <v>1</v>
+      </c>
+      <c r="D185" t="s">
+        <v>711</v>
+      </c>
+      <c r="E185" t="s">
+        <v>17</v>
+      </c>
+      <c r="F185" t="s">
+        <v>17</v>
+      </c>
+      <c r="G185" t="s">
+        <v>715</v>
+      </c>
+      <c r="H185" t="s">
+        <v>716</v>
+      </c>
+      <c r="I185">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>717</v>
+      </c>
+      <c r="B186" t="s">
+        <v>718</v>
+      </c>
+      <c r="C186">
+        <v>1</v>
+      </c>
+      <c r="D186" t="s">
+        <v>711</v>
+      </c>
+      <c r="E186" t="s">
+        <v>17</v>
+      </c>
+      <c r="F186" t="s">
+        <v>17</v>
+      </c>
+      <c r="G186" t="s">
+        <v>719</v>
+      </c>
+      <c r="H186" t="s">
+        <v>720</v>
+      </c>
+      <c r="I186">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>721</v>
+      </c>
+      <c r="B187" t="s">
+        <v>722</v>
+      </c>
+      <c r="C187">
+        <v>1</v>
+      </c>
+      <c r="D187" t="s">
+        <v>676</v>
+      </c>
+      <c r="E187" t="s">
+        <v>17</v>
+      </c>
+      <c r="F187" t="s">
+        <v>17</v>
+      </c>
+      <c r="G187" t="s">
+        <v>723</v>
+      </c>
+      <c r="H187" t="s">
+        <v>724</v>
+      </c>
+      <c r="I187">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>725</v>
+      </c>
+      <c r="B188" t="s">
+        <v>726</v>
+      </c>
+      <c r="C188">
+        <v>1</v>
+      </c>
+      <c r="D188" t="s">
+        <v>676</v>
+      </c>
+      <c r="E188" t="s">
+        <v>17</v>
+      </c>
+      <c r="F188" t="s">
+        <v>17</v>
+      </c>
+      <c r="G188" t="s">
+        <v>727</v>
+      </c>
+      <c r="H188" t="s">
+        <v>728</v>
+      </c>
+      <c r="I188">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>729</v>
+      </c>
+      <c r="B189" t="s">
+        <v>730</v>
+      </c>
+      <c r="C189">
+        <v>1</v>
+      </c>
+      <c r="D189" t="s">
+        <v>731</v>
+      </c>
+      <c r="E189" t="s">
+        <v>17</v>
+      </c>
+      <c r="F189" t="s">
+        <v>17</v>
+      </c>
+      <c r="G189" t="s">
+        <v>732</v>
+      </c>
+      <c r="H189" t="s">
+        <v>733</v>
+      </c>
+      <c r="I189">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>734</v>
+      </c>
+      <c r="B190" t="s">
+        <v>735</v>
+      </c>
+      <c r="C190">
+        <v>1</v>
+      </c>
+      <c r="D190" t="s">
+        <v>731</v>
+      </c>
+      <c r="E190" t="s">
+        <v>17</v>
+      </c>
+      <c r="F190" t="s">
+        <v>17</v>
+      </c>
+      <c r="G190" t="s">
+        <v>736</v>
+      </c>
+      <c r="H190" t="s">
+        <v>737</v>
+      </c>
+      <c r="I190">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>738</v>
+      </c>
+      <c r="B191" t="s">
+        <v>739</v>
+      </c>
+      <c r="C191">
+        <v>1</v>
+      </c>
+      <c r="D191" t="s">
+        <v>731</v>
+      </c>
+      <c r="E191" t="s">
+        <v>17</v>
+      </c>
+      <c r="F191" t="s">
+        <v>17</v>
+      </c>
+      <c r="G191" t="s">
+        <v>740</v>
+      </c>
+      <c r="H191" t="s">
+        <v>741</v>
+      </c>
+      <c r="I191">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>742</v>
+      </c>
+      <c r="B192" t="s">
+        <v>743</v>
+      </c>
+      <c r="C192">
+        <v>1</v>
+      </c>
+      <c r="D192" t="s">
+        <v>731</v>
+      </c>
+      <c r="E192" t="s">
+        <v>17</v>
+      </c>
+      <c r="F192" t="s">
+        <v>17</v>
+      </c>
+      <c r="G192" t="s">
+        <v>744</v>
+      </c>
+      <c r="H192" t="s">
+        <v>745</v>
+      </c>
+      <c r="I192">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>746</v>
+      </c>
+      <c r="B193" t="s">
+        <v>747</v>
+      </c>
+      <c r="C193">
+        <v>1</v>
+      </c>
+      <c r="D193" t="s">
+        <v>676</v>
+      </c>
+      <c r="E193" t="s">
+        <v>17</v>
+      </c>
+      <c r="F193" t="s">
+        <v>17</v>
+      </c>
+      <c r="G193" t="s">
+        <v>748</v>
+      </c>
+      <c r="H193" t="s">
+        <v>749</v>
+      </c>
+      <c r="I193">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>750</v>
+      </c>
+      <c r="B194" t="s">
+        <v>751</v>
+      </c>
+      <c r="C194">
+        <v>1</v>
+      </c>
+      <c r="D194" t="s">
+        <v>752</v>
+      </c>
+      <c r="E194" t="s">
+        <v>17</v>
+      </c>
+      <c r="F194" t="s">
+        <v>17</v>
+      </c>
+      <c r="G194" t="s">
+        <v>753</v>
+      </c>
+      <c r="H194" t="s">
+        <v>754</v>
+      </c>
+      <c r="I194">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>755</v>
+      </c>
+      <c r="B195" t="s">
+        <v>756</v>
+      </c>
+      <c r="C195">
+        <v>1</v>
+      </c>
+      <c r="D195" t="s">
+        <v>752</v>
+      </c>
+      <c r="E195" t="s">
+        <v>17</v>
+      </c>
+      <c r="F195" t="s">
+        <v>17</v>
+      </c>
+      <c r="G195" t="s">
+        <v>757</v>
+      </c>
+      <c r="H195" t="s">
+        <v>758</v>
+      </c>
+      <c r="I195">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>759</v>
+      </c>
+      <c r="B196" t="s">
+        <v>760</v>
+      </c>
+      <c r="C196">
+        <v>1</v>
+      </c>
+      <c r="D196" t="s">
+        <v>752</v>
+      </c>
+      <c r="E196" t="s">
+        <v>17</v>
+      </c>
+      <c r="F196" t="s">
+        <v>17</v>
+      </c>
+      <c r="G196" t="s">
+        <v>761</v>
+      </c>
+      <c r="H196" t="s">
+        <v>762</v>
+      </c>
+      <c r="I196">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>763</v>
+      </c>
+      <c r="B197" t="s">
+        <v>764</v>
+      </c>
+      <c r="C197">
+        <v>1</v>
+      </c>
+      <c r="D197" t="s">
+        <v>752</v>
+      </c>
+      <c r="E197" t="s">
+        <v>17</v>
+      </c>
+      <c r="F197" t="s">
+        <v>17</v>
+      </c>
+      <c r="G197" t="s">
+        <v>765</v>
+      </c>
+      <c r="H197" t="s">
+        <v>766</v>
+      </c>
+      <c r="I197">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>767</v>
+      </c>
+      <c r="B198" t="s">
+        <v>768</v>
+      </c>
+      <c r="C198">
+        <v>1</v>
+      </c>
+      <c r="D198" t="s">
+        <v>769</v>
+      </c>
+      <c r="E198" t="s">
+        <v>17</v>
+      </c>
+      <c r="F198" t="s">
+        <v>17</v>
+      </c>
+      <c r="G198" t="s">
+        <v>770</v>
+      </c>
+      <c r="H198" t="s">
+        <v>771</v>
+      </c>
+      <c r="I198">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>772</v>
+      </c>
+      <c r="B199" t="s">
+        <v>773</v>
+      </c>
+      <c r="C199">
+        <v>1</v>
+      </c>
+      <c r="D199" t="s">
+        <v>769</v>
+      </c>
+      <c r="E199" t="s">
+        <v>17</v>
+      </c>
+      <c r="F199" t="s">
+        <v>17</v>
+      </c>
+      <c r="G199" t="s">
+        <v>774</v>
+      </c>
+      <c r="H199" t="s">
+        <v>775</v>
+      </c>
+      <c r="I199">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>776</v>
+      </c>
+      <c r="B200" t="s">
+        <v>777</v>
+      </c>
+      <c r="C200">
+        <v>1</v>
+      </c>
+      <c r="D200" t="s">
+        <v>778</v>
+      </c>
+      <c r="E200" t="s">
+        <v>17</v>
+      </c>
+      <c r="F200" t="s">
+        <v>17</v>
+      </c>
+      <c r="G200" t="s">
+        <v>779</v>
+      </c>
+      <c r="H200" t="s">
+        <v>780</v>
+      </c>
+      <c r="I200">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>781</v>
+      </c>
+      <c r="B201" t="s">
+        <v>782</v>
+      </c>
+      <c r="C201">
+        <v>1</v>
+      </c>
+      <c r="D201" t="s">
+        <v>778</v>
+      </c>
+      <c r="E201" t="s">
+        <v>17</v>
+      </c>
+      <c r="F201" t="s">
+        <v>17</v>
+      </c>
+      <c r="G201" t="s">
+        <v>783</v>
+      </c>
+      <c r="H201" t="s">
+        <v>784</v>
+      </c>
+      <c r="I201">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>785</v>
+      </c>
+      <c r="B202" t="s">
+        <v>786</v>
+      </c>
+      <c r="C202">
+        <v>1</v>
+      </c>
+      <c r="D202" t="s">
+        <v>778</v>
+      </c>
+      <c r="E202" t="s">
+        <v>17</v>
+      </c>
+      <c r="F202" t="s">
+        <v>17</v>
+      </c>
+      <c r="G202" t="s">
+        <v>787</v>
+      </c>
+      <c r="H202" t="s">
+        <v>788</v>
+      </c>
+      <c r="I202">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>789</v>
+      </c>
+      <c r="B203" t="s">
+        <v>790</v>
+      </c>
+      <c r="C203">
+        <v>1</v>
+      </c>
+      <c r="D203" t="s">
+        <v>778</v>
+      </c>
+      <c r="E203" t="s">
+        <v>17</v>
+      </c>
+      <c r="F203" t="s">
+        <v>17</v>
+      </c>
+      <c r="G203" t="s">
+        <v>791</v>
+      </c>
+      <c r="H203" t="s">
+        <v>792</v>
+      </c>
+      <c r="I203">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>793</v>
+      </c>
+      <c r="B204" t="s">
+        <v>794</v>
+      </c>
+      <c r="C204">
+        <v>1</v>
+      </c>
+      <c r="D204" t="s">
+        <v>769</v>
+      </c>
+      <c r="E204" t="s">
+        <v>17</v>
+      </c>
+      <c r="F204" t="s">
+        <v>17</v>
+      </c>
+      <c r="G204" t="s">
+        <v>795</v>
+      </c>
+      <c r="H204" t="s">
+        <v>796</v>
+      </c>
+      <c r="I204">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>797</v>
+      </c>
+      <c r="B205" t="s">
+        <v>798</v>
+      </c>
+      <c r="C205">
+        <v>1</v>
+      </c>
+      <c r="D205" t="s">
+        <v>769</v>
+      </c>
+      <c r="E205" t="s">
+        <v>17</v>
+      </c>
+      <c r="F205" t="s">
+        <v>17</v>
+      </c>
+      <c r="G205" t="s">
+        <v>799</v>
+      </c>
+      <c r="H205" t="s">
+        <v>800</v>
+      </c>
+      <c r="I205">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>801</v>
+      </c>
+      <c r="B206" t="s">
+        <v>802</v>
+      </c>
+      <c r="C206">
+        <v>1</v>
+      </c>
+      <c r="D206" t="s">
+        <v>769</v>
+      </c>
+      <c r="E206" t="s">
+        <v>17</v>
+      </c>
+      <c r="F206" t="s">
+        <v>17</v>
+      </c>
+      <c r="G206" t="s">
+        <v>803</v>
+      </c>
+      <c r="H206" t="s">
+        <v>804</v>
+      </c>
+      <c r="I206">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>805</v>
+      </c>
+      <c r="B207" t="s">
+        <v>806</v>
+      </c>
+      <c r="C207">
+        <v>1</v>
+      </c>
+      <c r="D207" t="s">
+        <v>778</v>
+      </c>
+      <c r="E207" t="s">
+        <v>17</v>
+      </c>
+      <c r="F207" t="s">
+        <v>17</v>
+      </c>
+      <c r="G207" t="s">
+        <v>807</v>
+      </c>
+      <c r="H207" t="s">
+        <v>808</v>
+      </c>
+      <c r="I207">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>809</v>
+      </c>
+      <c r="B208" t="s">
+        <v>810</v>
+      </c>
+      <c r="C208">
+        <v>1</v>
+      </c>
+      <c r="D208" t="s">
+        <v>811</v>
+      </c>
+      <c r="E208" t="s">
+        <v>17</v>
+      </c>
+      <c r="F208" t="s">
+        <v>17</v>
+      </c>
+      <c r="G208" t="s">
+        <v>812</v>
+      </c>
+      <c r="H208" t="s">
+        <v>813</v>
+      </c>
+      <c r="I208">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>814</v>
+      </c>
+      <c r="B209" t="s">
+        <v>815</v>
+      </c>
+      <c r="C209">
+        <v>1</v>
+      </c>
+      <c r="D209" t="s">
+        <v>811</v>
+      </c>
+      <c r="E209" t="s">
+        <v>17</v>
+      </c>
+      <c r="F209" t="s">
+        <v>17</v>
+      </c>
+      <c r="G209" t="s">
+        <v>748</v>
+      </c>
+      <c r="H209" t="s">
+        <v>816</v>
+      </c>
+      <c r="I209">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>817</v>
+      </c>
+      <c r="B210" t="s">
+        <v>818</v>
+      </c>
+      <c r="C210">
+        <v>1</v>
+      </c>
+      <c r="D210" t="s">
+        <v>778</v>
+      </c>
+      <c r="E210" t="s">
+        <v>819</v>
+      </c>
+      <c r="F210" t="s">
+        <v>17</v>
+      </c>
+      <c r="G210" t="s">
+        <v>820</v>
+      </c>
+      <c r="H210" t="s">
+        <v>821</v>
+      </c>
+      <c r="I210">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>822</v>
+      </c>
+      <c r="B211" t="s">
+        <v>823</v>
+      </c>
+      <c r="C211">
+        <v>1</v>
+      </c>
+      <c r="D211" t="s">
+        <v>778</v>
+      </c>
+      <c r="E211" t="s">
+        <v>17</v>
+      </c>
+      <c r="F211" t="s">
+        <v>17</v>
+      </c>
+      <c r="G211" t="s">
+        <v>824</v>
+      </c>
+      <c r="H211" t="s">
+        <v>825</v>
+      </c>
+      <c r="I211">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>826</v>
+      </c>
+      <c r="B212" t="s">
+        <v>827</v>
+      </c>
+      <c r="C212">
+        <v>1</v>
+      </c>
+      <c r="D212" t="s">
+        <v>769</v>
+      </c>
+      <c r="E212" t="s">
+        <v>822</v>
+      </c>
+      <c r="F212" t="s">
+        <v>17</v>
+      </c>
+      <c r="G212" t="s">
+        <v>828</v>
+      </c>
+      <c r="H212" t="s">
+        <v>829</v>
+      </c>
+      <c r="I212">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>830</v>
+      </c>
+      <c r="B213" t="s">
+        <v>831</v>
+      </c>
+      <c r="C213">
+        <v>1</v>
+      </c>
+      <c r="D213" t="s">
+        <v>778</v>
+      </c>
+      <c r="E213" t="s">
+        <v>17</v>
+      </c>
+      <c r="F213" t="s">
+        <v>17</v>
+      </c>
+      <c r="G213" t="s">
+        <v>832</v>
+      </c>
+      <c r="H213" t="s">
+        <v>833</v>
+      </c>
+      <c r="I213">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>834</v>
+      </c>
+      <c r="B214" t="s">
+        <v>835</v>
+      </c>
+      <c r="C214">
+        <v>1</v>
+      </c>
+      <c r="D214" t="s">
+        <v>778</v>
+      </c>
+      <c r="E214" t="s">
+        <v>17</v>
+      </c>
+      <c r="F214" t="s">
+        <v>17</v>
+      </c>
+      <c r="G214" t="s">
+        <v>836</v>
+      </c>
+      <c r="H214" t="s">
+        <v>837</v>
+      </c>
+      <c r="I214">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>838</v>
+      </c>
+      <c r="B215" t="s">
+        <v>839</v>
+      </c>
+      <c r="C215">
+        <v>1</v>
+      </c>
+      <c r="D215" t="s">
+        <v>778</v>
+      </c>
+      <c r="E215" t="s">
+        <v>17</v>
+      </c>
+      <c r="F215" t="s">
+        <v>17</v>
+      </c>
+      <c r="G215" t="s">
+        <v>840</v>
+      </c>
+      <c r="H215" t="s">
+        <v>841</v>
+      </c>
+      <c r="I215">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>842</v>
+      </c>
+      <c r="B216" t="s">
+        <v>843</v>
+      </c>
+      <c r="C216">
+        <v>1</v>
+      </c>
+      <c r="D216" t="s">
+        <v>769</v>
+      </c>
+      <c r="E216" t="s">
+        <v>17</v>
+      </c>
+      <c r="F216" t="s">
+        <v>17</v>
+      </c>
+      <c r="G216" t="s">
+        <v>844</v>
+      </c>
+      <c r="H216" t="s">
+        <v>845</v>
+      </c>
+      <c r="I216">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>846</v>
+      </c>
+      <c r="B217" t="s">
+        <v>847</v>
+      </c>
+      <c r="C217">
+        <v>1</v>
+      </c>
+      <c r="D217" t="s">
+        <v>769</v>
+      </c>
+      <c r="E217" t="s">
+        <v>17</v>
+      </c>
+      <c r="F217" t="s">
+        <v>17</v>
+      </c>
+      <c r="G217" t="s">
+        <v>848</v>
+      </c>
+      <c r="H217" t="s">
+        <v>849</v>
+      </c>
+      <c r="I217">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>850</v>
+      </c>
+      <c r="B218" t="s">
+        <v>851</v>
+      </c>
+      <c r="C218">
+        <v>1</v>
+      </c>
+      <c r="D218" t="s">
+        <v>778</v>
+      </c>
+      <c r="E218" t="s">
+        <v>17</v>
+      </c>
+      <c r="F218" t="s">
+        <v>17</v>
+      </c>
+      <c r="G218" t="s">
+        <v>852</v>
+      </c>
+      <c r="H218" t="s">
+        <v>853</v>
+      </c>
+      <c r="I218">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>854</v>
+      </c>
+      <c r="B219" t="s">
+        <v>855</v>
+      </c>
+      <c r="C219">
+        <v>1</v>
+      </c>
+      <c r="D219" t="s">
+        <v>778</v>
+      </c>
+      <c r="E219" t="s">
+        <v>17</v>
+      </c>
+      <c r="F219" t="s">
+        <v>17</v>
+      </c>
+      <c r="G219" t="s">
+        <v>856</v>
+      </c>
+      <c r="H219" t="s">
+        <v>857</v>
+      </c>
+      <c r="I219">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>858</v>
+      </c>
+      <c r="B220" t="s">
+        <v>859</v>
+      </c>
+      <c r="C220">
+        <v>1</v>
+      </c>
+      <c r="D220" t="s">
+        <v>778</v>
+      </c>
+      <c r="E220" t="s">
+        <v>17</v>
+      </c>
+      <c r="F220" t="s">
+        <v>17</v>
+      </c>
+      <c r="G220" t="s">
+        <v>860</v>
+      </c>
+      <c r="H220" t="s">
+        <v>861</v>
+      </c>
+      <c r="I220">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>862</v>
+      </c>
+      <c r="B221" t="s">
+        <v>863</v>
+      </c>
+      <c r="C221">
+        <v>1</v>
+      </c>
+      <c r="D221" t="s">
+        <v>778</v>
+      </c>
+      <c r="E221" t="s">
+        <v>17</v>
+      </c>
+      <c r="F221" t="s">
+        <v>17</v>
+      </c>
+      <c r="G221" t="s">
+        <v>864</v>
+      </c>
+      <c r="H221" t="s">
+        <v>865</v>
+      </c>
+      <c r="I221">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>866</v>
+      </c>
+      <c r="B222" t="s">
+        <v>867</v>
+      </c>
+      <c r="C222">
+        <v>1</v>
+      </c>
+      <c r="D222" t="s">
+        <v>778</v>
+      </c>
+      <c r="E222" t="s">
+        <v>17</v>
+      </c>
+      <c r="F222" t="s">
+        <v>17</v>
+      </c>
+      <c r="G222" t="s">
+        <v>868</v>
+      </c>
+      <c r="H222" t="s">
+        <v>869</v>
+      </c>
+      <c r="I222">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>870</v>
+      </c>
+      <c r="B223" t="s">
+        <v>871</v>
+      </c>
+      <c r="C223">
+        <v>1</v>
+      </c>
+      <c r="D223" t="s">
+        <v>778</v>
+      </c>
+      <c r="E223" t="s">
+        <v>17</v>
+      </c>
+      <c r="F223" t="s">
+        <v>17</v>
+      </c>
+      <c r="G223" t="s">
+        <v>740</v>
+      </c>
+      <c r="H223" t="s">
+        <v>872</v>
+      </c>
+      <c r="I223">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>873</v>
+      </c>
+      <c r="B224" t="s">
+        <v>874</v>
+      </c>
+      <c r="C224">
+        <v>1</v>
+      </c>
+      <c r="D224" t="s">
+        <v>778</v>
+      </c>
+      <c r="E224" t="s">
+        <v>17</v>
+      </c>
+      <c r="F224" t="s">
+        <v>17</v>
+      </c>
+      <c r="G224" t="s">
+        <v>875</v>
+      </c>
+      <c r="H224" t="s">
+        <v>876</v>
+      </c>
+      <c r="I224">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>877</v>
+      </c>
+      <c r="B225" t="s">
+        <v>878</v>
+      </c>
+      <c r="C225">
+        <v>1</v>
+      </c>
+      <c r="D225" t="s">
+        <v>811</v>
+      </c>
+      <c r="E225" t="s">
+        <v>17</v>
+      </c>
+      <c r="F225" t="s">
+        <v>814</v>
+      </c>
+      <c r="G225" t="s">
+        <v>879</v>
+      </c>
+      <c r="H225" t="s">
+        <v>880</v>
+      </c>
+      <c r="I225">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>881</v>
+      </c>
+      <c r="B226" t="s">
+        <v>882</v>
+      </c>
+      <c r="C226">
+        <v>1</v>
+      </c>
+      <c r="D226" t="s">
+        <v>778</v>
+      </c>
+      <c r="E226" t="s">
+        <v>17</v>
+      </c>
+      <c r="F226" t="s">
+        <v>17</v>
+      </c>
+      <c r="G226" t="s">
+        <v>883</v>
+      </c>
+      <c r="H226" t="s">
+        <v>884</v>
+      </c>
+      <c r="I226">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>885</v>
+      </c>
+      <c r="B227" t="s">
+        <v>886</v>
+      </c>
+      <c r="C227">
+        <v>1</v>
+      </c>
+      <c r="D227" t="s">
+        <v>778</v>
+      </c>
+      <c r="E227" t="s">
+        <v>17</v>
+      </c>
+      <c r="F227" t="s">
+        <v>887</v>
+      </c>
+      <c r="G227" t="s">
+        <v>888</v>
+      </c>
+      <c r="H227" t="s">
+        <v>889</v>
+      </c>
+      <c r="I227">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>819</v>
+      </c>
+      <c r="B228" t="s">
+        <v>890</v>
+      </c>
+      <c r="C228">
+        <v>1</v>
+      </c>
+      <c r="D228" t="s">
+        <v>778</v>
+      </c>
+      <c r="E228" t="s">
+        <v>17</v>
+      </c>
+      <c r="F228" t="s">
+        <v>891</v>
+      </c>
+      <c r="G228" t="s">
+        <v>892</v>
+      </c>
+      <c r="H228" t="s">
+        <v>893</v>
+      </c>
+      <c r="I228">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>894</v>
+      </c>
+      <c r="B229" t="s">
+        <v>895</v>
+      </c>
+      <c r="C229">
+        <v>1</v>
+      </c>
+      <c r="D229" t="s">
+        <v>778</v>
+      </c>
+      <c r="E229" t="s">
+        <v>17</v>
+      </c>
+      <c r="F229" t="s">
+        <v>17</v>
+      </c>
+      <c r="G229" t="s">
+        <v>896</v>
+      </c>
+      <c r="H229" t="s">
+        <v>897</v>
+      </c>
+      <c r="I229">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>898</v>
+      </c>
+      <c r="B230" t="s">
+        <v>899</v>
+      </c>
+      <c r="C230">
+        <v>1</v>
+      </c>
+      <c r="D230" t="s">
+        <v>778</v>
+      </c>
+      <c r="E230" t="s">
+        <v>17</v>
+      </c>
+      <c r="F230" t="s">
+        <v>17</v>
+      </c>
+      <c r="G230" t="s">
+        <v>900</v>
+      </c>
+      <c r="H230" t="s">
+        <v>901</v>
+      </c>
+      <c r="I230">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>902</v>
+      </c>
+      <c r="B231" t="s">
+        <v>903</v>
+      </c>
+      <c r="C231">
+        <v>1</v>
+      </c>
+      <c r="D231" t="s">
+        <v>778</v>
+      </c>
+      <c r="E231" t="s">
+        <v>17</v>
+      </c>
+      <c r="F231" t="s">
+        <v>17</v>
+      </c>
+      <c r="G231" t="s">
+        <v>740</v>
+      </c>
+      <c r="H231" t="s">
+        <v>904</v>
+      </c>
+      <c r="I231">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>905</v>
+      </c>
+      <c r="B232" t="s">
+        <v>906</v>
+      </c>
+      <c r="C232">
+        <v>1</v>
+      </c>
+      <c r="D232" t="s">
+        <v>811</v>
+      </c>
+      <c r="E232" t="s">
+        <v>17</v>
+      </c>
+      <c r="F232" t="s">
+        <v>17</v>
+      </c>
+      <c r="G232" t="s">
+        <v>907</v>
+      </c>
+      <c r="H232" t="s">
+        <v>908</v>
+      </c>
+      <c r="I232">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>909</v>
+      </c>
+      <c r="B233" t="s">
+        <v>910</v>
+      </c>
+      <c r="C233">
+        <v>1</v>
+      </c>
+      <c r="D233" t="s">
+        <v>778</v>
+      </c>
+      <c r="E233" t="s">
+        <v>17</v>
+      </c>
+      <c r="F233" t="s">
+        <v>17</v>
+      </c>
+      <c r="G233" t="s">
+        <v>911</v>
+      </c>
+      <c r="H233" t="s">
+        <v>912</v>
+      </c>
+      <c r="I233">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>913</v>
+      </c>
+      <c r="B234" t="s">
+        <v>914</v>
+      </c>
+      <c r="C234">
+        <v>1</v>
+      </c>
+      <c r="D234" t="s">
+        <v>778</v>
+      </c>
+      <c r="E234" t="s">
+        <v>17</v>
+      </c>
+      <c r="F234" t="s">
+        <v>17</v>
+      </c>
+      <c r="G234" t="s">
+        <v>915</v>
+      </c>
+      <c r="H234" t="s">
+        <v>916</v>
+      </c>
+      <c r="I234">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>917</v>
+      </c>
+      <c r="B235" t="s">
+        <v>918</v>
+      </c>
+      <c r="C235">
+        <v>1</v>
+      </c>
+      <c r="D235" t="s">
+        <v>778</v>
+      </c>
+      <c r="E235" t="s">
+        <v>17</v>
+      </c>
+      <c r="F235" t="s">
+        <v>17</v>
+      </c>
+      <c r="G235" t="s">
+        <v>919</v>
+      </c>
+      <c r="H235" t="s">
+        <v>920</v>
+      </c>
+      <c r="I235">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>921</v>
+      </c>
+      <c r="B236" t="s">
+        <v>922</v>
+      </c>
+      <c r="C236">
+        <v>1</v>
+      </c>
+      <c r="D236" t="s">
+        <v>778</v>
+      </c>
+      <c r="E236" t="s">
+        <v>17</v>
+      </c>
+      <c r="F236" t="s">
+        <v>17</v>
+      </c>
+      <c r="G236" t="s">
+        <v>923</v>
+      </c>
+      <c r="H236" t="s">
+        <v>924</v>
+      </c>
+      <c r="I236">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>925</v>
+      </c>
+      <c r="B237" t="s">
+        <v>926</v>
+      </c>
+      <c r="C237">
+        <v>1</v>
+      </c>
+      <c r="D237" t="s">
+        <v>927</v>
+      </c>
+      <c r="E237" t="s">
+        <v>17</v>
+      </c>
+      <c r="F237" t="s">
+        <v>17</v>
+      </c>
+      <c r="G237" t="s">
+        <v>928</v>
+      </c>
+      <c r="H237" t="s">
+        <v>929</v>
+      </c>
+      <c r="I237">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>930</v>
+      </c>
+      <c r="B238" t="s">
+        <v>931</v>
+      </c>
+      <c r="C238">
+        <v>1</v>
+      </c>
+      <c r="D238" t="s">
+        <v>927</v>
+      </c>
+      <c r="E238" t="s">
+        <v>17</v>
+      </c>
+      <c r="F238" t="s">
+        <v>17</v>
+      </c>
+      <c r="G238" t="s">
+        <v>932</v>
+      </c>
+      <c r="H238" t="s">
+        <v>933</v>
+      </c>
+      <c r="I238">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>934</v>
+      </c>
+      <c r="B239" t="s">
+        <v>935</v>
+      </c>
+      <c r="C239">
+        <v>1</v>
+      </c>
+      <c r="D239" t="s">
+        <v>778</v>
+      </c>
+      <c r="E239" t="s">
+        <v>17</v>
+      </c>
+      <c r="F239" t="s">
+        <v>17</v>
+      </c>
+      <c r="G239" t="s">
+        <v>936</v>
+      </c>
+      <c r="H239" t="s">
+        <v>937</v>
+      </c>
+      <c r="I239">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>938</v>
+      </c>
+      <c r="B240" t="s">
+        <v>939</v>
+      </c>
+      <c r="C240">
+        <v>1</v>
+      </c>
+      <c r="D240" t="s">
+        <v>778</v>
+      </c>
+      <c r="E240" t="s">
+        <v>17</v>
+      </c>
+      <c r="F240" t="s">
+        <v>17</v>
+      </c>
+      <c r="G240" t="s">
+        <v>740</v>
+      </c>
+      <c r="H240" t="s">
+        <v>940</v>
+      </c>
+      <c r="I240">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>941</v>
+      </c>
+      <c r="B241" t="s">
+        <v>942</v>
+      </c>
+      <c r="C241">
+        <v>1</v>
+      </c>
+      <c r="D241" t="s">
+        <v>778</v>
+      </c>
+      <c r="E241" t="s">
+        <v>17</v>
+      </c>
+      <c r="F241" t="s">
+        <v>17</v>
+      </c>
+      <c r="G241" t="s">
+        <v>943</v>
+      </c>
+      <c r="H241" t="s">
+        <v>944</v>
+      </c>
+      <c r="I241">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>945</v>
+      </c>
+      <c r="B242" t="s">
+        <v>946</v>
+      </c>
+      <c r="C242">
+        <v>1</v>
+      </c>
+      <c r="D242" t="s">
+        <v>778</v>
+      </c>
+      <c r="E242" t="s">
+        <v>17</v>
+      </c>
+      <c r="F242" t="s">
+        <v>17</v>
+      </c>
+      <c r="G242" t="s">
+        <v>947</v>
+      </c>
+      <c r="H242" t="s">
+        <v>948</v>
+      </c>
+      <c r="I242">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>949</v>
+      </c>
+      <c r="B243" t="s">
+        <v>950</v>
+      </c>
+      <c r="C243">
+        <v>1</v>
+      </c>
+      <c r="D243" t="s">
+        <v>778</v>
+      </c>
+      <c r="E243" t="s">
+        <v>17</v>
+      </c>
+      <c r="F243" t="s">
+        <v>17</v>
+      </c>
+      <c r="G243" t="s">
+        <v>951</v>
+      </c>
+      <c r="H243" t="s">
+        <v>728</v>
+      </c>
+      <c r="I243">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>952</v>
+      </c>
+      <c r="B244" t="s">
+        <v>953</v>
+      </c>
+      <c r="C244">
+        <v>1</v>
+      </c>
+      <c r="D244" t="s">
+        <v>769</v>
+      </c>
+      <c r="E244" t="s">
+        <v>17</v>
+      </c>
+      <c r="F244" t="s">
+        <v>17</v>
+      </c>
+      <c r="G244" t="s">
+        <v>774</v>
+      </c>
+      <c r="H244" t="s">
+        <v>954</v>
+      </c>
+      <c r="I244">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>955</v>
+      </c>
+      <c r="B245" t="s">
+        <v>956</v>
+      </c>
+      <c r="C245">
+        <v>1</v>
+      </c>
+      <c r="D245" t="s">
+        <v>778</v>
+      </c>
+      <c r="E245" t="s">
+        <v>17</v>
+      </c>
+      <c r="F245" t="s">
+        <v>17</v>
+      </c>
+      <c r="G245" t="s">
+        <v>957</v>
+      </c>
+      <c r="H245" t="s">
+        <v>958</v>
+      </c>
+      <c r="I245">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>959</v>
+      </c>
+      <c r="B246" t="s">
+        <v>960</v>
+      </c>
+      <c r="C246">
+        <v>1</v>
+      </c>
+      <c r="D246" t="s">
+        <v>811</v>
+      </c>
+      <c r="E246" t="s">
+        <v>17</v>
+      </c>
+      <c r="F246" t="s">
+        <v>17</v>
+      </c>
+      <c r="G246" t="s">
+        <v>961</v>
+      </c>
+      <c r="H246" t="s">
+        <v>962</v>
+      </c>
+      <c r="I246">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>963</v>
+      </c>
+      <c r="B247" t="s">
+        <v>964</v>
+      </c>
+      <c r="C247">
+        <v>1</v>
+      </c>
+      <c r="D247" t="s">
+        <v>778</v>
+      </c>
+      <c r="E247" t="s">
+        <v>17</v>
+      </c>
+      <c r="F247" t="s">
+        <v>17</v>
+      </c>
+      <c r="G247" t="s">
+        <v>965</v>
+      </c>
+      <c r="H247" t="s">
+        <v>966</v>
+      </c>
+      <c r="I247">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>967</v>
+      </c>
+      <c r="B248" t="s">
+        <v>968</v>
+      </c>
+      <c r="C248">
+        <v>1</v>
+      </c>
+      <c r="D248" t="s">
+        <v>778</v>
+      </c>
+      <c r="E248" t="s">
+        <v>17</v>
+      </c>
+      <c r="F248" t="s">
+        <v>17</v>
+      </c>
+      <c r="G248" t="s">
+        <v>969</v>
+      </c>
+      <c r="H248" t="s">
+        <v>970</v>
+      </c>
+      <c r="I248">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>971</v>
+      </c>
+      <c r="B249" t="s">
+        <v>972</v>
+      </c>
+      <c r="C249">
+        <v>1</v>
+      </c>
+      <c r="D249" t="s">
+        <v>769</v>
+      </c>
+      <c r="E249" t="s">
+        <v>17</v>
+      </c>
+      <c r="F249" t="s">
+        <v>17</v>
+      </c>
+      <c r="G249" t="s">
+        <v>973</v>
+      </c>
+      <c r="H249" t="s">
+        <v>974</v>
+      </c>
+      <c r="I249">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>975</v>
+      </c>
+      <c r="B250" t="s">
+        <v>976</v>
+      </c>
+      <c r="C250" s="3">
+        <v>46024</v>
+      </c>
+      <c r="D250" t="s">
+        <v>811</v>
+      </c>
+      <c r="E250" t="s">
+        <v>17</v>
+      </c>
+      <c r="F250" t="s">
+        <v>17</v>
+      </c>
+      <c r="G250" t="s">
+        <v>977</v>
+      </c>
+      <c r="H250" t="s">
+        <v>978</v>
+      </c>
+      <c r="I250">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>979</v>
+      </c>
+      <c r="B251" t="s">
+        <v>980</v>
+      </c>
+      <c r="C251" s="3">
+        <v>46024</v>
+      </c>
+      <c r="D251" t="s">
+        <v>811</v>
+      </c>
+      <c r="E251" t="s">
+        <v>17</v>
+      </c>
+      <c r="F251" t="s">
+        <v>17</v>
+      </c>
+      <c r="G251" t="s">
+        <v>981</v>
+      </c>
+      <c r="H251" t="s">
+        <v>982</v>
+      </c>
+      <c r="I251">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>983</v>
+      </c>
+      <c r="B252" t="s">
+        <v>984</v>
+      </c>
+      <c r="C252" s="3">
+        <v>46024</v>
+      </c>
+      <c r="D252" t="s">
+        <v>985</v>
+      </c>
+      <c r="E252" t="s">
+        <v>17</v>
+      </c>
+      <c r="F252" t="s">
+        <v>17</v>
+      </c>
+      <c r="G252" t="s">
+        <v>986</v>
+      </c>
+      <c r="H252" t="s">
+        <v>987</v>
+      </c>
+      <c r="I252">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A253" t="s">
+        <v>988</v>
+      </c>
+      <c r="B253" t="s">
+        <v>989</v>
+      </c>
+      <c r="C253" s="3">
+        <v>46024</v>
+      </c>
+      <c r="D253" t="s">
+        <v>778</v>
+      </c>
+      <c r="E253" t="s">
+        <v>17</v>
+      </c>
+      <c r="F253" t="s">
+        <v>17</v>
+      </c>
+      <c r="G253" t="s">
+        <v>990</v>
+      </c>
+      <c r="H253" t="s">
+        <v>991</v>
+      </c>
+      <c r="I253">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>